<commit_message>
Use manuscript figures and processed-data labels
</commit_message>
<xml_diff>
--- a/data/public/public_data_catalog.xlsx
+++ b/data/public/public_data_catalog.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="World Bank FAO" sheetId="1" r:id="Rc94a6948c26541f0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MOA Annual" sheetId="2" r:id="Rcd9d2f4182d04a57"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Source Catalog" sheetId="3" r:id="R19084b2b4ca24a81"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Notes" sheetId="4" r:id="Rc11e18618de548ca"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="World Bank FAO" sheetId="1" r:id="Rca514eb3c19e4662"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MOA Annual" sheetId="2" r:id="Rfa2b091653944a39"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Source Catalog" sheetId="3" r:id="R349029b6d04c46e8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Notes" sheetId="4" r:id="R256f1dec6cda4fca"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -3769,6 +3769,7 @@
     <x:col min="7" max="7" width="34" hidden="0" customWidth="1"/>
     <x:col min="8" max="8" width="48" hidden="0" customWidth="1"/>
     <x:col min="9" max="9" width="15" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="70" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="30" customHeight="1">
@@ -3799,7 +3800,7 @@
       <x:c r="I1" s="30" t="str">
         <x:v>retrieved_on</x:v>
       </x:c>
-      <x:c r="J1" t="str">
+      <x:c r="J1" s="30" t="str">
         <x:v>notes</x:v>
       </x:c>
     </x:row>
@@ -3831,7 +3832,7 @@
       <x:c r="I2" s="26" t="str">
         <x:v>2026-07-23</x:v>
       </x:c>
-      <x:c r="J2" t="str">
+      <x:c r="J2" s="26" t="str">
         <x:v>National series; not a substitute for the missing 31-province coefficient matrix.</x:v>
       </x:c>
     </x:row>
@@ -3863,7 +3864,7 @@
       <x:c r="I3" s="26" t="str">
         <x:v>2026-07-23</x:v>
       </x:c>
-      <x:c r="J3" t="str">
+      <x:c r="J3" s="26" t="str">
         <x:v>National series; not a substitute for the missing 31-province coefficient matrix.</x:v>
       </x:c>
     </x:row>
@@ -3895,7 +3896,7 @@
       <x:c r="I4" s="26" t="str">
         <x:v>2026-07-23</x:v>
       </x:c>
-      <x:c r="J4" t="str">
+      <x:c r="J4" s="26" t="str">
         <x:v>National series; not a substitute for the missing 31-province coefficient matrix.</x:v>
       </x:c>
     </x:row>
@@ -3927,7 +3928,7 @@
       <x:c r="I5" s="26" t="str">
         <x:v>2026-07-23</x:v>
       </x:c>
-      <x:c r="J5" t="str">
+      <x:c r="J5" s="26" t="str">
         <x:v>2017 is an attachment-only legacy DOC and 2018 was not available as an accessible official HTML page; neither is silently interpolated.</x:v>
       </x:c>
     </x:row>
@@ -3959,7 +3960,7 @@
       <x:c r="I6" s="26" t="str">
         <x:v>2026-07-23</x:v>
       </x:c>
-      <x:c r="J6" t="str">
+      <x:c r="J6" s="26" t="str">
         <x:v>2017 is an attachment-only legacy DOC and 2018 was not available as an accessible official HTML page; neither is silently interpolated.</x:v>
       </x:c>
     </x:row>
@@ -3991,7 +3992,7 @@
       <x:c r="I7" s="26" t="str">
         <x:v>2026-07-23</x:v>
       </x:c>
-      <x:c r="J7" t="str">
+      <x:c r="J7" s="26" t="str">
         <x:v>2017 is an attachment-only legacy DOC and 2018 was not available as an accessible official HTML page; neither is silently interpolated.</x:v>
       </x:c>
     </x:row>
@@ -4023,7 +4024,7 @@
       <x:c r="I8" s="26" t="str">
         <x:v>2026-07-23</x:v>
       </x:c>
-      <x:c r="J8" t="str">
+      <x:c r="J8" s="26" t="str">
         <x:v>2017 is an attachment-only legacy DOC and 2018 was not available as an accessible official HTML page; neither is silently interpolated.</x:v>
       </x:c>
     </x:row>
@@ -4055,7 +4056,7 @@
       <x:c r="I9" s="26" t="str">
         <x:v>2026-07-23</x:v>
       </x:c>
-      <x:c r="J9" t="str">
+      <x:c r="J9" s="26" t="str">
         <x:v>2017 is an attachment-only legacy DOC and 2018 was not available as an accessible official HTML page; neither is silently interpolated.</x:v>
       </x:c>
     </x:row>
@@ -4087,7 +4088,7 @@
       <x:c r="I10" s="26" t="str">
         <x:v>2026-07-23</x:v>
       </x:c>
-      <x:c r="J10" t="str">
+      <x:c r="J10" s="26" t="str">
         <x:v>2017 is an attachment-only legacy DOC and 2018 was not available as an accessible official HTML page; neither is silently interpolated.</x:v>
       </x:c>
     </x:row>
@@ -4119,7 +4120,7 @@
       <x:c r="I11" s="26" t="str">
         <x:v>2026-07-23</x:v>
       </x:c>
-      <x:c r="J11" t="str">
+      <x:c r="J11" s="26" t="str">
         <x:v>2017 is an attachment-only legacy DOC and 2018 was not available as an accessible official HTML page; neither is silently interpolated.</x:v>
       </x:c>
     </x:row>
@@ -4149,7 +4150,7 @@
       <x:c r="I12" s="26" t="str">
         <x:v>2026-07-23</x:v>
       </x:c>
-      <x:c r="J12" t="str">
+      <x:c r="J12" s="26" t="str">
         <x:v>Not redistributed because a reliable machine-readable download could not be obtained from the official endpoint.</x:v>
       </x:c>
     </x:row>
@@ -4179,7 +4180,7 @@
       <x:c r="I13" s="26" t="str">
         <x:v>2026-07-23</x:v>
       </x:c>
-      <x:c r="J13" t="str">
+      <x:c r="J13" s="26" t="str">
         <x:v>The official statistical-system page explains that annual results are published through the yearbook.</x:v>
       </x:c>
     </x:row>
@@ -4254,10 +4255,10 @@
     </x:row>
     <x:row r="8" ht="34" customHeight="1">
       <x:c r="A8" s="26" t="str">
-        <x:v>Article reconstruction</x:v>
+        <x:v>数据标识 / Data label</x:v>
       </x:c>
       <x:c r="B8" s="26" t="str">
-        <x:v>Figures 2-10 remain calibrated reconstructions, not author run logs</x:v>
+        <x:v>经过处理的数据 (processed data); figure CSVs are derived from disclosed anchors, not author run logs</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="34" customHeight="1">

</xml_diff>